<commit_message>
Updated ETH_grids_kan10 model - 2026-06-18 23:16
</commit_message>
<xml_diff>
--- a/VerveStacks_GHA_grids_kan10/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GHA_grids_kan10/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GHA_grids_kan10\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8A22BA2-4C4B-4DFF-8240-6034B9335835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA64059B-BA86-4AE1-BDA6-1FCB0236C1F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -849,22 +849,58 @@
     <t>connecting solar to buses in cluster 7</t>
   </si>
   <si>
+    <t>distr_solelc_spv_GHA_014</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 14</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_GHA_003</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_GHA_005</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 5</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_GHA_015</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 15</t>
   </si>
   <si>
+    <t>distr_solelc_spv_GHA_013</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 13</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_GHA_006</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_solelc_spv_GHA_008</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 8</t>
+  </si>
+  <si>
     <t>distr_solelc_spv_GHA_002</t>
   </si>
   <si>
     <t>connecting solar to buses in cluster 2</t>
   </si>
   <si>
-    <t>distr_solelc_spv_GHA_013</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 13</t>
+    <t>distr_solelc_spv_GHA_009</t>
+  </si>
+  <si>
+    <t>connecting solar to buses in cluster 9</t>
   </si>
   <si>
     <t>distr_solelc_spv_GHA_012</t>
@@ -897,42 +933,6 @@
     <t>connecting solar to buses in cluster 16</t>
   </si>
   <si>
-    <t>distr_solelc_spv_GHA_009</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 9</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_GHA_006</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_GHA_008</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_GHA_014</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 14</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_GHA_003</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_solelc_spv_GHA_005</t>
-  </si>
-  <si>
-    <t>connecting solar to buses in cluster 5</t>
-  </si>
-  <si>
     <t>comm-in</t>
   </si>
   <si>
@@ -948,13 +948,25 @@
     <t>e_w1069597794-330_GHA</t>
   </si>
   <si>
+    <t>e_w674068904-225_GHA</t>
+  </si>
+  <si>
+    <t>e_r15772152-330_GHA,e_w1069597794-330_GHA</t>
+  </si>
+  <si>
     <t>e_w672526714-330_GHA,e_w674068904-225_GHA</t>
   </si>
   <si>
+    <t>e_w674068904-225_GHA,e_w1155380911-330_GHA</t>
+  </si>
+  <si>
+    <t>e_w282578857-330_GHA,e_w1069597794-330_GHA</t>
+  </si>
+  <si>
     <t>e_r15772152-330_GHA,e_w1069597794-330_GHA,e_w930744195-225_GHA</t>
   </si>
   <si>
-    <t>e_w674068904-225_GHA,e_w1155380911-330_GHA</t>
+    <t>e_w1155380911-330_GHA,e_r15772152-330_GHA,e_w1069597794-330_GHA</t>
   </si>
   <si>
     <t>e_w1155380911-330_GHA,e_r15772152-330_GHA</t>
@@ -969,16 +981,10 @@
     <t>e_w282578857-330_GHA</t>
   </si>
   <si>
-    <t>e_w1155380911-330_GHA,e_r15772152-330_GHA,e_w1069597794-330_GHA</t>
-  </si>
-  <si>
-    <t>e_r15772152-330_GHA,e_w1069597794-330_GHA</t>
-  </si>
-  <si>
-    <t>e_w282578857-330_GHA,e_w1069597794-330_GHA</t>
-  </si>
-  <si>
-    <t>e_w674068904-225_GHA</t>
+    <t>distr_wonelc_won_GHA_010</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 10</t>
   </si>
   <si>
     <t>distr_wonelc_won_GHA_007</t>
@@ -987,6 +993,42 @@
     <t>connecting wind onshore to buses in cluster 7</t>
   </si>
   <si>
+    <t>distr_wonelc_won_GHA_001</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_GHA_004</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_GHA_009</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 9</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_GHA_006</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 6</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_GHA_003</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 3</t>
+  </si>
+  <si>
+    <t>distr_wonelc_won_GHA_005</t>
+  </si>
+  <si>
+    <t>connecting wind onshore to buses in cluster 5</t>
+  </si>
+  <si>
     <t>distr_wonelc_won_GHA_002</t>
   </si>
   <si>
@@ -999,79 +1041,73 @@
     <t>connecting wind onshore to buses in cluster 8</t>
   </si>
   <si>
-    <t>distr_wonelc_won_GHA_003</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 3</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_GHA_010</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 10</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_GHA_001</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_GHA_006</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 6</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_GHA_005</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 5</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_GHA_004</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_wonelc_won_GHA_009</t>
-  </si>
-  <si>
-    <t>connecting wind onshore to buses in cluster 9</t>
+    <t>elc_won_GHA_010</t>
   </si>
   <si>
     <t>elc_won_GHA_007</t>
   </si>
   <si>
+    <t>elc_won_GHA_001</t>
+  </si>
+  <si>
+    <t>e_w282578857-330_GHA,e_w672526714-330_GHA</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_004</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_009</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_006</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_003</t>
+  </si>
+  <si>
+    <t>elc_won_GHA_005</t>
+  </si>
+  <si>
     <t>elc_won_GHA_002</t>
   </si>
   <si>
     <t>elc_won_GHA_008</t>
   </si>
   <si>
-    <t>elc_won_GHA_003</t>
-  </si>
-  <si>
-    <t>elc_won_GHA_010</t>
-  </si>
-  <si>
-    <t>elc_won_GHA_001</t>
-  </si>
-  <si>
-    <t>e_w282578857-330_GHA,e_w672526714-330_GHA</t>
-  </si>
-  <si>
-    <t>elc_won_GHA_006</t>
-  </si>
-  <si>
-    <t>elc_won_GHA_005</t>
-  </si>
-  <si>
-    <t>elc_won_GHA_004</t>
-  </si>
-  <si>
-    <t>elc_won_GHA_009</t>
+    <t>distr_wofelc_wof_GHA_008</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 8</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_GHA_002</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 2</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_GHA_004</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 4</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_GHA_007</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 7</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_GHA_001</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 1</t>
+  </si>
+  <si>
+    <t>distr_wofelc_wof_GHA_009</t>
+  </si>
+  <si>
+    <t>connecting wind offshore to buses in cluster 9</t>
   </si>
   <si>
     <t>distr_wofelc_wof_GHA_006</t>
@@ -1080,30 +1116,6 @@
     <t>connecting wind offshore to buses in cluster 6</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_GHA_002</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 2</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_GHA_004</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 4</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_GHA_001</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 1</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_GHA_009</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 9</t>
-  </si>
-  <si>
     <t>distr_wofelc_wof_GHA_003</t>
   </si>
   <si>
@@ -1122,36 +1134,30 @@
     <t>connecting wind offshore to buses in cluster 10</t>
   </si>
   <si>
-    <t>distr_wofelc_wof_GHA_008</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 8</t>
-  </si>
-  <si>
-    <t>distr_wofelc_wof_GHA_007</t>
-  </si>
-  <si>
-    <t>connecting wind offshore to buses in cluster 7</t>
+    <t>elc_wof_GHA_008</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_002</t>
+  </si>
+  <si>
+    <t>e_w672526714-330_GHA</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_004</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_007</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_001</t>
+  </si>
+  <si>
+    <t>elc_wof_GHA_009</t>
   </si>
   <si>
     <t>elc_wof_GHA_006</t>
   </si>
   <si>
-    <t>elc_wof_GHA_002</t>
-  </si>
-  <si>
-    <t>e_w672526714-330_GHA</t>
-  </si>
-  <si>
-    <t>elc_wof_GHA_004</t>
-  </si>
-  <si>
-    <t>elc_wof_GHA_001</t>
-  </si>
-  <si>
-    <t>elc_wof_GHA_009</t>
-  </si>
-  <si>
     <t>elc_wof_GHA_003</t>
   </si>
   <si>
@@ -1159,12 +1165,6 @@
   </si>
   <si>
     <t>elc_wof_GHA_010</t>
-  </si>
-  <si>
-    <t>elc_wof_GHA_008</t>
-  </si>
-  <si>
-    <t>elc_wof_GHA_007</t>
   </si>
   <si>
     <t>e_won_GHA_001</t>
@@ -3308,7 +3308,7 @@
         <v>50</v>
       </c>
       <c r="V28" s="147" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -6109,7 +6109,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44F5B2A7-C530-44CC-A571-44E3E962A60E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBAD19E0-7F9E-4D6C-BADD-022A15651C00}">
   <dimension ref="B9:BD27"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6389,10 +6389,10 @@
         <v>272</v>
       </c>
       <c r="AO11">
-        <v>0.98997046923979071</v>
+        <v>0.99474449552139477</v>
       </c>
       <c r="AP11">
-        <v>183.87473060383624</v>
+        <v>96.350915441096063</v>
       </c>
       <c r="AR11" t="s">
         <v>231</v>
@@ -6422,13 +6422,13 @@
         <v>335</v>
       </c>
       <c r="BB11" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="BC11">
-        <v>0.99602973628442149</v>
+        <v>0.9976147902706346</v>
       </c>
       <c r="BD11">
-        <v>72.788168118939723</v>
+        <v>43.728845038365712</v>
       </c>
     </row>
     <row r="12" spans="2:56">
@@ -6532,13 +6532,13 @@
         <v>305</v>
       </c>
       <c r="AN12" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="AO12">
-        <v>0.99636177435061024</v>
+        <v>0.98997046923979071</v>
       </c>
       <c r="AP12">
-        <v>66.700803572145503</v>
+        <v>183.87473060383624</v>
       </c>
       <c r="AR12" t="s">
         <v>231</v>
@@ -6678,13 +6678,13 @@
         <v>306</v>
       </c>
       <c r="AN13" t="s">
-        <v>270</v>
+        <v>307</v>
       </c>
       <c r="AO13">
-        <v>0.99014192318757677</v>
+        <v>0.99623091337490355</v>
       </c>
       <c r="AP13">
-        <v>180.73140822775915</v>
+        <v>69.099921460101669</v>
       </c>
       <c r="AR13" t="s">
         <v>231</v>
@@ -6785,16 +6785,16 @@
         <v>240</v>
       </c>
       <c r="Y14" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="Z14" t="s">
         <v>273</v>
       </c>
       <c r="AA14">
-        <v>0.99772747376800408</v>
+        <v>0.99828853709516652</v>
       </c>
       <c r="AB14">
-        <v>41.662980919925118</v>
+        <v>31.376819921947806</v>
       </c>
       <c r="AD14" t="s">
         <v>231</v>
@@ -6821,16 +6821,16 @@
         <v>290</v>
       </c>
       <c r="AM14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AN14" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="AO14">
-        <v>0.99392958354540772</v>
+        <v>0.99056449392208212</v>
       </c>
       <c r="AP14">
-        <v>111.29096833419247</v>
+        <v>172.98427809516085</v>
       </c>
       <c r="AR14" t="s">
         <v>231</v>
@@ -6863,10 +6863,10 @@
         <v>283</v>
       </c>
       <c r="BC14">
-        <v>0.99676013971200861</v>
+        <v>0.99691010026270699</v>
       </c>
       <c r="BD14">
-        <v>59.397438613176035</v>
+        <v>56.648161850371878</v>
       </c>
     </row>
     <row r="15" spans="2:56">
@@ -6931,16 +6931,16 @@
         <v>242</v>
       </c>
       <c r="Y15" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Z15" t="s">
         <v>274</v>
       </c>
       <c r="AA15">
-        <v>0.99144816104289235</v>
+        <v>0.99414237783753501</v>
       </c>
       <c r="AB15">
-        <v>156.78371421363983</v>
+        <v>107.38973964519224</v>
       </c>
       <c r="AD15" t="s">
         <v>231</v>
@@ -6967,16 +6967,16 @@
         <v>292</v>
       </c>
       <c r="AM15" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AN15" t="s">
         <v>272</v>
       </c>
       <c r="AO15">
-        <v>0.99474449552139477</v>
+        <v>0.99243615939349938</v>
       </c>
       <c r="AP15">
-        <v>96.350915441096063</v>
+        <v>138.67041111917737</v>
       </c>
       <c r="AR15" t="s">
         <v>231</v>
@@ -7006,13 +7006,13 @@
         <v>340</v>
       </c>
       <c r="BB15" t="s">
-        <v>310</v>
+        <v>273</v>
       </c>
       <c r="BC15">
-        <v>0.99433636733393604</v>
+        <v>0.99676013971200861</v>
       </c>
       <c r="BD15">
-        <v>103.83326554450551</v>
+        <v>59.397438613176035</v>
       </c>
     </row>
     <row r="16" spans="2:56">
@@ -7077,16 +7077,16 @@
         <v>244</v>
       </c>
       <c r="Y16" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="Z16" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="AA16">
-        <v>0.99639529182713771</v>
+        <v>0.9971980297205405</v>
       </c>
       <c r="AB16">
-        <v>66.086316502475782</v>
+        <v>51.369455123424352</v>
       </c>
       <c r="AD16" t="s">
         <v>231</v>
@@ -7113,16 +7113,16 @@
         <v>294</v>
       </c>
       <c r="AM16" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="AN16" t="s">
-        <v>310</v>
+        <v>270</v>
       </c>
       <c r="AO16">
-        <v>0.99623091337490355</v>
+        <v>0.99564542867887518</v>
       </c>
       <c r="AP16">
-        <v>69.099921460101669</v>
+        <v>79.833807553954642</v>
       </c>
       <c r="AR16" t="s">
         <v>231</v>
@@ -7152,13 +7152,13 @@
         <v>341</v>
       </c>
       <c r="BB16" t="s">
-        <v>337</v>
+        <v>307</v>
       </c>
       <c r="BC16">
-        <v>0.99905788912759763</v>
+        <v>0.99433636733393604</v>
       </c>
       <c r="BD16">
-        <v>17.272032660709108</v>
+        <v>103.83326554450551</v>
       </c>
     </row>
     <row r="17" spans="2:56">
@@ -7223,16 +7223,16 @@
         <v>246</v>
       </c>
       <c r="Y17" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="Z17" t="s">
         <v>275</v>
       </c>
       <c r="AA17">
-        <v>0.99450622481426521</v>
+        <v>0.99772747376800408</v>
       </c>
       <c r="AB17">
-        <v>100.71921173847173</v>
+        <v>41.662980919925118</v>
       </c>
       <c r="AD17" t="s">
         <v>231</v>
@@ -7262,13 +7262,13 @@
         <v>311</v>
       </c>
       <c r="AN17" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="AO17">
-        <v>0.99564542867887518</v>
+        <v>0.99392958354540772</v>
       </c>
       <c r="AP17">
-        <v>79.833807553954642</v>
+        <v>111.29096833419247</v>
       </c>
       <c r="AR17" t="s">
         <v>231</v>
@@ -7298,13 +7298,13 @@
         <v>342</v>
       </c>
       <c r="BB17" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="BC17">
-        <v>0.9953748577774012</v>
+        <v>0.99602973628442149</v>
       </c>
       <c r="BD17">
-        <v>84.794274080978198</v>
+        <v>72.788168118939723</v>
       </c>
     </row>
     <row r="18" spans="2:56">
@@ -7369,16 +7369,16 @@
         <v>248</v>
       </c>
       <c r="Y18" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="Z18" t="s">
         <v>276</v>
       </c>
       <c r="AA18">
-        <v>0.99453161000209944</v>
+        <v>0.99639529182713771</v>
       </c>
       <c r="AB18">
-        <v>100.25381662817612</v>
+        <v>66.086316502475782</v>
       </c>
       <c r="AD18" t="s">
         <v>231</v>
@@ -7408,7 +7408,7 @@
         <v>312</v>
       </c>
       <c r="AN18" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="AO18">
         <v>0.99594979093510827</v>
@@ -7444,13 +7444,13 @@
         <v>343</v>
       </c>
       <c r="BB18" t="s">
-        <v>279</v>
+        <v>337</v>
       </c>
       <c r="BC18">
-        <v>0.99418918260895706</v>
+        <v>0.99905788912759763</v>
       </c>
       <c r="BD18">
-        <v>106.53165216912117</v>
+        <v>17.272032660709108</v>
       </c>
     </row>
     <row r="19" spans="2:56">
@@ -7515,16 +7515,16 @@
         <v>250</v>
       </c>
       <c r="Y19" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="Z19" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="AA19">
-        <v>0.99575843323891533</v>
+        <v>0.9973925893911626</v>
       </c>
       <c r="AB19">
-        <v>77.762057286552078</v>
+        <v>47.802527828685051</v>
       </c>
       <c r="AD19" t="s">
         <v>231</v>
@@ -7554,13 +7554,13 @@
         <v>313</v>
       </c>
       <c r="AN19" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="AO19">
-        <v>0.99056449392208212</v>
+        <v>0.99636177435061024</v>
       </c>
       <c r="AP19">
-        <v>172.98427809516085</v>
+        <v>66.700803572145503</v>
       </c>
       <c r="AR19" t="s">
         <v>231</v>
@@ -7590,13 +7590,13 @@
         <v>344</v>
       </c>
       <c r="BB19" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="BC19">
-        <v>0.9976147902706346</v>
+        <v>0.9953748577774012</v>
       </c>
       <c r="BD19">
-        <v>43.728845038365712</v>
+        <v>84.794274080978198</v>
       </c>
     </row>
     <row r="20" spans="2:56">
@@ -7661,16 +7661,16 @@
         <v>252</v>
       </c>
       <c r="Y20" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="Z20" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="AA20">
-        <v>0.99497862751910049</v>
+        <v>0.99127486150655841</v>
       </c>
       <c r="AB20">
-        <v>92.058495483157941</v>
+        <v>159.96087237976209</v>
       </c>
       <c r="AD20" t="s">
         <v>231</v>
@@ -7700,13 +7700,13 @@
         <v>314</v>
       </c>
       <c r="AN20" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="AO20">
-        <v>0.99243615939349938</v>
+        <v>0.99014192318757677</v>
       </c>
       <c r="AP20">
-        <v>138.67041111917737</v>
+        <v>180.73140822775915</v>
       </c>
       <c r="AR20" t="s">
         <v>231</v>
@@ -7736,13 +7736,13 @@
         <v>345</v>
       </c>
       <c r="BB20" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="BC20">
-        <v>0.99691010026270699</v>
+        <v>0.99418918260895706</v>
       </c>
       <c r="BD20">
-        <v>56.648161850371878</v>
+        <v>106.53165216912117</v>
       </c>
     </row>
     <row r="21" spans="2:56">
@@ -7807,16 +7807,16 @@
         <v>254</v>
       </c>
       <c r="Y21" t="s">
-        <v>228</v>
+        <v>214</v>
       </c>
       <c r="Z21" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="AA21">
-        <v>0.99551622817514029</v>
+        <v>0.99144816104289235</v>
       </c>
       <c r="AB21">
-        <v>82.202483455762263</v>
+        <v>156.78371421363983</v>
       </c>
     </row>
     <row r="22" spans="2:56">
@@ -7884,7 +7884,7 @@
         <v>221</v>
       </c>
       <c r="Z22" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="AA22">
         <v>0.99184937635213322</v>
@@ -7955,16 +7955,16 @@
         <v>258</v>
       </c>
       <c r="Y23" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="Z23" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="AA23">
-        <v>0.9973925893911626</v>
+        <v>0.99450622481426521</v>
       </c>
       <c r="AB23">
-        <v>47.802527828685051</v>
+        <v>100.71921173847173</v>
       </c>
     </row>
     <row r="24" spans="2:56">
@@ -8029,16 +8029,16 @@
         <v>260</v>
       </c>
       <c r="Y24" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="Z24" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="AA24">
-        <v>0.99127486150655841</v>
+        <v>0.99453161000209944</v>
       </c>
       <c r="AB24">
-        <v>159.96087237976209</v>
+        <v>100.25381662817612</v>
       </c>
     </row>
     <row r="25" spans="2:56">
@@ -8103,16 +8103,16 @@
         <v>262</v>
       </c>
       <c r="Y25" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="Z25" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="AA25">
-        <v>0.99828853709516652</v>
+        <v>0.99575843323891533</v>
       </c>
       <c r="AB25">
-        <v>31.376819921947806</v>
+        <v>77.762057286552078</v>
       </c>
     </row>
     <row r="26" spans="2:56">
@@ -8177,16 +8177,16 @@
         <v>264</v>
       </c>
       <c r="Y26" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="Z26" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AA26">
-        <v>0.99414237783753501</v>
+        <v>0.99497862751910049</v>
       </c>
       <c r="AB26">
-        <v>107.38973964519224</v>
+        <v>92.058495483157941</v>
       </c>
     </row>
     <row r="27" spans="2:56">
@@ -8251,16 +8251,16 @@
         <v>266</v>
       </c>
       <c r="Y27" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="Z27" t="s">
-        <v>270</v>
+        <v>283</v>
       </c>
       <c r="AA27">
-        <v>0.9971980297205405</v>
+        <v>0.99551622817514029</v>
       </c>
       <c r="AB27">
-        <v>51.369455123424352</v>
+        <v>82.202483455762263</v>
       </c>
     </row>
   </sheetData>
@@ -8269,7 +8269,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F239BD15-2279-4E3E-BDFB-E8DB2A05D029}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9065E114-BCFB-438D-A34C-72F17806C79D}">
   <dimension ref="B9:Z20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8381,7 +8381,7 @@
         <v>346</v>
       </c>
       <c r="K11" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="L11">
         <v>0.23559225287113886</v>
@@ -8414,7 +8414,7 @@
         <v>366</v>
       </c>
       <c r="X11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="Y11">
         <v>0.68774999999999997</v>
@@ -8449,7 +8449,7 @@
         <v>348</v>
       </c>
       <c r="K12" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="L12">
         <v>1.6401923188479914</v>
@@ -8517,7 +8517,7 @@
         <v>350</v>
       </c>
       <c r="K13" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="L13">
         <v>2.4594087827359172</v>
@@ -8550,7 +8550,7 @@
         <v>370</v>
       </c>
       <c r="X13" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="Y13">
         <v>1.1617500000000001</v>
@@ -8585,7 +8585,7 @@
         <v>352</v>
       </c>
       <c r="K14" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="L14">
         <v>1.7739898665785649</v>
@@ -8686,7 +8686,7 @@
         <v>374</v>
       </c>
       <c r="X15" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="Y15">
         <v>1.2817499999999999</v>
@@ -8721,7 +8721,7 @@
         <v>356</v>
       </c>
       <c r="K16" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L16">
         <v>0.27801729674041986</v>
@@ -8754,7 +8754,7 @@
         <v>376</v>
       </c>
       <c r="X16" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="Y16">
         <v>3.0644999999999998</v>
@@ -8789,7 +8789,7 @@
         <v>358</v>
       </c>
       <c r="K17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L17">
         <v>0.41527678836292919</v>
@@ -8822,7 +8822,7 @@
         <v>378</v>
       </c>
       <c r="X17" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="Y17">
         <v>0.44024999999999997</v>
@@ -8857,7 +8857,7 @@
         <v>360</v>
       </c>
       <c r="K18" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="L18">
         <v>0.33510531500553531</v>
@@ -8890,7 +8890,7 @@
         <v>380</v>
       </c>
       <c r="X18" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="Y18">
         <v>3.351</v>
@@ -8925,7 +8925,7 @@
         <v>362</v>
       </c>
       <c r="K19" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="L19">
         <v>0.28254977119147401</v>
@@ -8958,7 +8958,7 @@
         <v>382</v>
       </c>
       <c r="X19" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="Y19">
         <v>3.87825</v>
@@ -8993,7 +8993,7 @@
         <v>364</v>
       </c>
       <c r="K20" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="L20">
         <v>0.1973305247660169</v>
@@ -9026,7 +9026,7 @@
         <v>384</v>
       </c>
       <c r="X20" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="Y20">
         <v>7.8750000000000001E-2</v>
@@ -9041,7 +9041,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C211B4C4-D19E-40D6-986D-45A861253DC6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21BA7179-B57A-4C81-ACBC-1668737D82C0}">
   <dimension ref="B9:S128"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>